<commit_message>
Update internship targets spreadsheet with new data
</commit_message>
<xml_diff>
--- a/Summer_2027_Internship_Targets_Koa_Shen_Updated.xlsx
+++ b/Summer_2027_Internship_Targets_Koa_Shen_Updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://slac-my.sharepoint.com/personal/koashen_slac_stanford_edu/Documents/portfolio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{8D6F4D6C-2762-48A4-842D-913E3512EB4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E6795C0-E892-4784-803E-E6945EC637F8}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{8D6F4D6C-2762-48A4-842D-913E3512EB4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC21FB98-8EFF-43F5-B2D1-84FF40BBACE8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{9540BDC1-F339-4E20-9435-EAA7DBCBFB18}"/>
   </bookViews>
@@ -4026,7 +4026,7 @@
         <v>54</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>55</v>
+        <v>671</v>
       </c>
       <c r="N4" s="10"/>
       <c r="O4" s="6"/>
@@ -4120,7 +4120,7 @@
         <v>54</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>69</v>
+        <v>671</v>
       </c>
       <c r="N6" s="10"/>
       <c r="O6" s="7">
@@ -4169,7 +4169,7 @@
         <v>54</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>55</v>
+        <v>671</v>
       </c>
       <c r="N7" s="10"/>
       <c r="O7" s="6"/>

</xml_diff>